<commit_message>
Update warehouse_gui_server: GUI/서버 최신화 + admin_gui·데이터 추가
- warehouse_gui_v2.py: 점유 해제(release_hold)·선점 확인 로직 추가
- warehouse_server_v2.py: 입고(inbound) API·품목 검색·release_hold 처리 추가
- admin_gui.py: 신규 추가 (실시간 재고 모니터링/로그)
- 데이터 베이스.xlsx, 사용자1주문.xlsx, 사용자2주문.xlsx 갱신

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/warehouse_gui_server/데이터 베이스.xlsx
+++ b/warehouse_gui_server/데이터 베이스.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11835" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 

</xml_diff>